<commit_message>
feat: integrate Phase 2 components into existing pages
- EscrowStatus + DeliveryVerification into TransactionPage (lazy-loaded)
- MultiChannelSupport replaces SuntrexSupportChat FAB in App.jsx
- Bulk import sidebar link in SIDEBAR_SELL + DashboardRouter mapping
- Fix DeliveryTrackerPage: remove unused react-i18next import
- Regenerate XLSX offer template

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/suntrex-offer-template.xlsx
+++ b/public/templates/suntrex-offer-template.xlsx
@@ -399,15 +399,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I4"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="38.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="8.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,25 +441,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SUN2000-10KTL-M2</v>
+        <v>SUN2000-10KTL</v>
       </c>
       <c r="B2" t="str">
-        <v>Huawei SUN2000-10KTL-M2 Onduleur</v>
+        <v>Huawei SUN2000-10KTL-M2</v>
       </c>
       <c r="C2" t="str">
         <v>Huawei</v>
       </c>
       <c r="D2">
-        <v>1850</v>
+        <v>1250</v>
       </c>
       <c r="E2">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H2" t="str">
         <v>DE</v>
@@ -470,25 +470,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SUN-12K-SG04LP3</v>
+        <v>DEYE-12K-SG04</v>
       </c>
       <c r="B3" t="str">
-        <v>Deye SUN-12K Hybrid Inverter</v>
+        <v>Deye SUN-12K-SG04LP3-EU</v>
       </c>
       <c r="C3" t="str">
         <v>Deye</v>
       </c>
       <c r="D3">
-        <v>1420</v>
+        <v>980</v>
       </c>
       <c r="E3">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H3" t="str">
         <v>NL</v>
@@ -499,25 +499,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>HVS-5.1</v>
+        <v>BYD-HVS-7.7</v>
       </c>
       <c r="B4" t="str">
-        <v>BYD Battery-Box HVS 5.1 kWh</v>
+        <v>BYD Battery-Box Premium HVS 7.7</v>
       </c>
       <c r="C4" t="str">
         <v>BYD</v>
       </c>
       <c r="D4">
-        <v>2100</v>
+        <v>3200</v>
       </c>
       <c r="E4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H4" t="str">
         <v>FR</v>

</xml_diff>